<commit_message>
Report Suite: companion-video deltas applied locally
7 tester-facing edits (nav anchors, PV not-only-Parts, customer-card Sales
Representative label, toggle path) + 13 notes-only annotations + Q5 appended
to the Chris sheet + SPEC-WATCH updated; 0 adds/deletes, tally 465;
deliverables regenerated, id-map 465/465 re-merged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/report-suite/PO-Questions-Chris-ReportSuite-TechPlan_2026-07-30.xlsx
+++ b/build/report-suite/PO-Questions-Chris-ReportSuite-TechPlan_2026-07-30.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,33 @@
       </c>
       <c r="F7" s="3" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>How far does "the full word Representative" go? (added 2026-07-30 after your companion video)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>In your companion video you asked us to always write out the full word "Representative" instead of the short "Rep", and you specifically corrected the customer card label to "Sales Representative" (we have updated our checks for that). But some smaller labels still use the short form by design today: the box on the work order where the sales person is picked is called "Sales Rep", and the assignments download is called "Sales Rep Assignments" (its file and one of its columns also say "Sales Rep").</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Should those smaller labels also spell out the full word, or can they keep the short form?</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>A) Every label everywhere uses the full word "Representative" - including the work order box and the assignments download with its file and columns.
+B) Only the report name and the customer card use the full word; the smaller "Sales Rep" labels can stay as they are.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -625,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -754,6 +781,26 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SBR-WO-01 (C30310); SBR-WO-02 (C30311); SBR-ASGN-01 (C30292); SBR-ASGN-02 (C30293)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Source: companion video 2026-07-30 C15 (09:41-10:10 no-short-forms ruling; 10:53-11:12 customer-card correction applied as FIRM to SBR-WO-06 C30315). Spec still says "Sales Rep" for the WO selector (S19-R1/R8) + the Assignments export name/header/filename (S15). Chris demonstrated the WO dropdown WITHOUT flagging its label, so the small labels were NOT flipped on the principle alone.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>A -&gt; flip the "Sales Rep" labels in the four cases (WO selector label/accessible name; export dialog entry, filename, CSV header) to the full word + spec pages updated. B -&gt; cases stand as authored. Either way VIU-confirm live.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>